<commit_message>
removed tenant name in rentroll template
</commit_message>
<xml_diff>
--- a/myapp/src/assets/Asset72_Rent_Roll_Template.xlsx
+++ b/myapp/src/assets/Asset72_Rent_Roll_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aneeshsai.m\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sriya.m\Documents\Realestate_Frontend\myapp\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66308C00-F9DA-49E1-9935-A0A4466E926F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FB395A0-2084-46D3-82E0-6C8A699FBF3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rent Roll Upload" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Property Name</t>
   </si>
@@ -29,9 +29,6 @@
   </si>
   <si>
     <t>Sq Ft</t>
-  </si>
-  <si>
-    <t>Tenant Name</t>
   </si>
   <si>
     <t>Lease Start Date</t>
@@ -404,7 +401,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -416,24 +413,22 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>6</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="J1" s="1"/>
     </row>
   </sheetData>
   <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" sqref="C2:F2 C3:F3 C4:F4 C5:F5 C6:F6 C7:F7 C8:F8 C9:F9 C10:F10 C11:F11 C12:F12 C13:F13 C14:F14 C15:F15 C16:F16 C17:F17 C18:F18 C19:F19 C20:F20 C21:F21 C22:F22 C23:F23 C24:F24 C25:F25 C26:F26 C27:F27 C28:F28 C29:F29 C30:F30 C31:F31 C32:F32 C33:F33 C34:F34 C35:F35 C36:F36 C37:F37 C38:F38 C39:F39 C40:F40 C41:F41 C42:F42 C43:F43 C44:F44 C45:F45 C46:F46 C47:F47 C48:F48 C49:F49 C50:F50 C51:F51 C52:F52 C53:F53 C54:F54 C55:F55 C56:F56 C57:F57 C58:F58 C59:F59 C60:F60 C61:F61 C62:F62 C63:F63 C64:F64 C65:F65 C66:F66 C67:F67 C68:F68 C69:F69 C70:F70 C71:F71 C72:F72 C73:F73 C74:F74 C75:F75 C76:F76 C77:F77 C78:F78 C79:F79 C80:F80 C81:F81 C82:F82 C83:F83 C84:F84 C85:F85 C86:F86 C87:F87 C88:F88 C89:F89 C90:F90 C91:F91 C92:F92 C93:F93 C94:F94 C95:F95 C96:F96 C97:F97 C98:F98 C99:F99 C100:F100 C101:F101 C102:F102 C103:F103 C104:F104 C105:F105 C106:F106 C107:F107 C108:F108 C109:F109 C110:F110 C111:F111 C112:F112 C113:F113 C114:F114 C115:F115 C116:F116 C117:F117 C118:F118 C119:F119 C120:F120 C121:F121 C122:F122 C123:F123 C124:F124 C125:F125 C126:F126 C127:F127 C128:F128 C129:F129 C130:F130 C131:F131 C132:F132 C133:F133 C134:F134 C135:F135 C136:F136 C137:F137 C138:F138 C139:F139 C140:F140 C141:F141 C142:F142 C143:F143 C144:F144 C145:F145 C146:F146 C147:F147 C148:F148 C149:F149" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="C2:F149" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Studio,1BR,2BR,3BR,Retail,Office"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>